<commit_message>
Corregir Excel a carta horizontal y retirar firma del tesorero
</commit_message>
<xml_diff>
--- a/portal/contributions-template.xlsx
+++ b/portal/contributions-template.xlsx
@@ -354,7 +354,7 @@
       <row>1</row>
       <rowOff>28575</rowOff>
     </from>
-    <ext cx="1200150" cy="1200150"/>
+    <ext cx="1066800" cy="1066800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="2922ec0d-1a34-49b8-8372-01fbffbfc1d4"/>
@@ -612,27 +612,27 @@
   <sheetPr>
     <tabColor rgb="FF25543C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
-    <col width="26" customWidth="1" style="11" min="1" max="1"/>
-    <col width="14" customWidth="1" style="11" min="2" max="2"/>
-    <col width="10" customWidth="1" style="11" min="3" max="3"/>
-    <col width="14" customWidth="1" style="11" min="4" max="4"/>
-    <col width="15" customWidth="1" style="11" min="5" max="5"/>
-    <col width="25" customWidth="1" style="11" min="6" max="6"/>
+    <col width="28" customWidth="1" style="11" min="1" max="1"/>
+    <col width="18" customWidth="1" style="11" min="2" max="2"/>
+    <col width="14" customWidth="1" style="11" min="3" max="3"/>
+    <col width="16" customWidth="1" style="11" min="4" max="4"/>
+    <col width="18" customWidth="1" style="11" min="5" max="5"/>
+    <col width="28" customWidth="1" style="11" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="11">
+    <row r="1" ht="16" customHeight="1" s="11">
       <c r="A1" s="16" t="inlineStr">
         <is>
           <t>LA QUINIELA FISCALIZADA</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="21" customHeight="1" s="11">
+    <row r="2" ht="18" customHeight="1" s="11">
       <c r="A2" s="19" t="n"/>
       <c r="B2" s="15" t="inlineStr">
         <is>
@@ -640,10 +640,10 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="21" customHeight="1" s="11">
+    <row r="3" ht="18" customHeight="1" s="11">
       <c r="A3" s="19" t="n"/>
     </row>
-    <row r="4" ht="18" customHeight="1" s="11">
+    <row r="4" ht="15" customHeight="1" s="11">
       <c r="A4" s="19" t="n"/>
       <c r="B4" s="10" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="21" customHeight="1" s="11">
+    <row r="5" ht="17" customHeight="1" s="11">
       <c r="A5" s="19" t="n"/>
       <c r="B5" s="19" t="inlineStr">
         <is>
@@ -659,7 +659,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="21" customHeight="1" s="11">
+    <row r="6" ht="18" customHeight="1" s="11">
       <c r="A6" s="19" t="n"/>
       <c r="B6" s="19" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="E6" s="12" t="n"/>
     </row>
-    <row r="7" ht="6" customHeight="1" s="11">
+    <row r="7" ht="5" customHeight="1" s="11">
       <c r="A7" s="19" t="n"/>
       <c r="B7" s="19" t="n"/>
       <c r="C7" s="19" t="n"/>
@@ -684,7 +684,7 @@
       <c r="E7" s="19" t="n"/>
       <c r="F7" s="19" t="n"/>
     </row>
-    <row r="8" ht="18" customHeight="1" s="11">
+    <row r="8" ht="15" customHeight="1" s="11">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>RECIBIDO (MXN)</t>
@@ -701,7 +701,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="23" customHeight="1" s="11">
+    <row r="9" ht="20" customHeight="1" s="11">
       <c r="A9" s="22">
         <f>SUM(D12:D27)</f>
         <v/>
@@ -715,14 +715,14 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="28" customHeight="1" s="11">
+    <row r="10" ht="21" customHeight="1" s="11">
       <c r="A10" s="14" t="inlineStr">
         <is>
           <t>En «Recibido», selecciona ✓ o ✗ en la PC, o marca la casilla a mano. Vacía = sin confirmar.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="28" customHeight="1" s="11">
+    <row r="11" ht="24" customHeight="1" s="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Participante</t>
@@ -740,7 +740,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Importe (MXN)</t>
+          <t>Importe</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -754,7 +754,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1" s="11">
+    <row r="12" ht="18" customHeight="1" s="11">
       <c r="A12" s="4" t="n"/>
       <c r="B12" s="6" t="n"/>
       <c r="C12" s="5" t="n"/>
@@ -765,7 +765,7 @@
       <c r="E12" s="8" t="n"/>
       <c r="F12" s="9" t="n"/>
     </row>
-    <row r="13" ht="24" customHeight="1" s="11">
+    <row r="13" ht="18" customHeight="1" s="11">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="6" t="n"/>
       <c r="C13" s="5" t="n"/>
@@ -776,7 +776,7 @@
       <c r="E13" s="8" t="n"/>
       <c r="F13" s="9" t="n"/>
     </row>
-    <row r="14" ht="24" customHeight="1" s="11">
+    <row r="14" ht="18" customHeight="1" s="11">
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="6" t="n"/>
       <c r="C14" s="5" t="n"/>
@@ -787,7 +787,7 @@
       <c r="E14" s="8" t="n"/>
       <c r="F14" s="9" t="n"/>
     </row>
-    <row r="15" ht="24" customHeight="1" s="11">
+    <row r="15" ht="18" customHeight="1" s="11">
       <c r="A15" s="4" t="n"/>
       <c r="B15" s="6" t="n"/>
       <c r="C15" s="5" t="n"/>
@@ -798,7 +798,7 @@
       <c r="E15" s="8" t="n"/>
       <c r="F15" s="9" t="n"/>
     </row>
-    <row r="16" ht="24" customHeight="1" s="11">
+    <row r="16" ht="18" customHeight="1" s="11">
       <c r="A16" s="4" t="n"/>
       <c r="B16" s="6" t="n"/>
       <c r="C16" s="5" t="n"/>
@@ -809,7 +809,7 @@
       <c r="E16" s="8" t="n"/>
       <c r="F16" s="9" t="n"/>
     </row>
-    <row r="17" ht="24" customHeight="1" s="11">
+    <row r="17" ht="18" customHeight="1" s="11">
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="6" t="n"/>
       <c r="C17" s="5" t="n"/>
@@ -820,7 +820,7 @@
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="9" t="n"/>
     </row>
-    <row r="18" ht="24" customHeight="1" s="11">
+    <row r="18" ht="18" customHeight="1" s="11">
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="6" t="n"/>
       <c r="C18" s="5" t="n"/>
@@ -831,7 +831,7 @@
       <c r="E18" s="8" t="n"/>
       <c r="F18" s="9" t="n"/>
     </row>
-    <row r="19" ht="24" customHeight="1" s="11">
+    <row r="19" ht="18" customHeight="1" s="11">
       <c r="A19" s="4" t="n"/>
       <c r="B19" s="6" t="n"/>
       <c r="C19" s="5" t="n"/>
@@ -842,7 +842,7 @@
       <c r="E19" s="8" t="n"/>
       <c r="F19" s="9" t="n"/>
     </row>
-    <row r="20" ht="24" customHeight="1" s="11">
+    <row r="20" ht="18" customHeight="1" s="11">
       <c r="A20" s="4" t="n"/>
       <c r="B20" s="6" t="n"/>
       <c r="C20" s="5" t="n"/>
@@ -853,7 +853,7 @@
       <c r="E20" s="8" t="n"/>
       <c r="F20" s="9" t="n"/>
     </row>
-    <row r="21" ht="24" customHeight="1" s="11">
+    <row r="21" ht="18" customHeight="1" s="11">
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="6" t="n"/>
       <c r="C21" s="5" t="n"/>
@@ -864,7 +864,7 @@
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="9" t="n"/>
     </row>
-    <row r="22" ht="24" customHeight="1" s="11">
+    <row r="22" ht="18" customHeight="1" s="11">
       <c r="A22" s="4" t="n"/>
       <c r="B22" s="6" t="n"/>
       <c r="C22" s="5" t="n"/>
@@ -875,7 +875,7 @@
       <c r="E22" s="8" t="n"/>
       <c r="F22" s="9" t="n"/>
     </row>
-    <row r="23" ht="24" customHeight="1" s="11">
+    <row r="23" ht="18" customHeight="1" s="11">
       <c r="A23" s="4" t="n"/>
       <c r="B23" s="6" t="n"/>
       <c r="C23" s="5" t="n"/>
@@ -886,7 +886,7 @@
       <c r="E23" s="8" t="n"/>
       <c r="F23" s="9" t="n"/>
     </row>
-    <row r="24" ht="24" customHeight="1" s="11">
+    <row r="24" ht="18" customHeight="1" s="11">
       <c r="A24" s="4" t="n"/>
       <c r="B24" s="6" t="n"/>
       <c r="C24" s="5" t="n"/>
@@ -897,7 +897,7 @@
       <c r="E24" s="8" t="n"/>
       <c r="F24" s="9" t="n"/>
     </row>
-    <row r="25" ht="24" customHeight="1" s="11">
+    <row r="25" ht="18" customHeight="1" s="11">
       <c r="A25" s="4" t="n"/>
       <c r="B25" s="6" t="n"/>
       <c r="C25" s="5" t="n"/>
@@ -908,7 +908,7 @@
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="9" t="n"/>
     </row>
-    <row r="26" ht="24" customHeight="1" s="11">
+    <row r="26" ht="18" customHeight="1" s="11">
       <c r="A26" s="4" t="n"/>
       <c r="B26" s="6" t="n"/>
       <c r="C26" s="5" t="n"/>
@@ -919,7 +919,7 @@
       <c r="E26" s="8" t="n"/>
       <c r="F26" s="9" t="n"/>
     </row>
-    <row r="27" ht="24" customHeight="1" s="11">
+    <row r="27" ht="18" customHeight="1" s="11">
       <c r="A27" s="4" t="n"/>
       <c r="B27" s="6" t="n"/>
       <c r="C27" s="5" t="n"/>
@@ -930,7 +930,7 @@
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="9" t="n"/>
     </row>
-    <row r="28" ht="6" customHeight="1" s="11">
+    <row r="28" ht="4" customHeight="1" s="11">
       <c r="A28" s="19" t="n"/>
       <c r="B28" s="19" t="n"/>
       <c r="C28" s="19" t="n"/>
@@ -938,7 +938,7 @@
       <c r="E28" s="19" t="n"/>
       <c r="F28" s="19" t="n"/>
     </row>
-    <row r="29" ht="18" customHeight="1" s="11">
+    <row r="29" ht="16" customHeight="1" s="11">
       <c r="A29" s="20" t="inlineStr">
         <is>
           <t>✓ Recibido     ✗ Pendiente     Vacía: sin confirmar</t>
@@ -947,7 +947,7 @@
       <c r="E29" s="19" t="n"/>
       <c r="F29" s="19" t="n"/>
     </row>
-    <row r="30" ht="22" customHeight="1" s="11">
+    <row r="30" ht="17" customHeight="1" s="11">
       <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Los cambios en Excel no se guardan en la plataforma.</t>
@@ -956,16 +956,12 @@
       <c r="E30" s="19" t="n"/>
       <c r="F30" s="19" t="n"/>
     </row>
-    <row r="31" ht="25" customHeight="1" s="11">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>Firma del tesorero: __________________________________</t>
-        </is>
-      </c>
+    <row r="31" ht="20" customHeight="1" s="11">
+      <c r="A31" s="13" t="n"/>
       <c r="E31" s="19" t="n"/>
       <c r="F31" s="19" t="n"/>
     </row>
-    <row r="32" ht="15" customHeight="1" s="11">
+    <row r="32" ht="12" customHeight="1" s="11">
       <c r="A32" s="23" t="inlineStr">
         <is>
           <t>quiniela-fiscalizada.up.railway.app</t>
@@ -1009,7 +1005,7 @@
   </dataValidations>
   <printOptions horizontalCentered="1" verticalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
-  <pageSetup orientation="portrait" paperSize="1" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Usar Montserrat en los Excel de aportaciones
</commit_message>
<xml_diff>
--- a/portal/contributions-template.xlsx
+++ b/portal/contributions-template.xlsx
@@ -13,7 +13,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Aportaciones'!$1:$11</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Aportaciones'!$A$1:$F$32</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -29,79 +29,79 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FF142B30"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
+      <family val="2"/>
+      <color rgb="FF142B30"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
       <family val="2"/>
       <b val="1"/>
       <color rgb="FF142B30"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <b val="1"/>
       <color rgb="FF25543C"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <b val="1"/>
       <color rgb="FF25543C"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <b val="1"/>
       <color rgb="FF25543C"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <color rgb="FF59705E"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <b val="1"/>
       <color rgb="FF25543C"/>
       <sz val="20"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <color rgb="FF25543C"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <color rgb="FF59705E"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <color rgb="FF142B30"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Montserrat"/>
       <family val="2"/>
       <color rgb="FF25543C"/>
       <sz val="9"/>
@@ -178,38 +178,38 @@
   </cellStyleXfs>
   <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -221,7 +221,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -230,7 +230,7 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -252,6 +252,7 @@
   <dxfs count="2">
     <dxf>
       <font>
+        <name val="Montserrat"/>
         <b val="1"/>
         <color rgb="FF8F453B"/>
       </font>
@@ -263,6 +264,7 @@
     </dxf>
     <dxf>
       <font>
+        <name val="Montserrat"/>
         <b val="1"/>
         <color rgb="FF25543C"/>
       </font>
@@ -756,8 +758,8 @@
     </row>
     <row r="12" ht="18" customHeight="1" s="11">
       <c r="A12" s="4" t="n"/>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="6" t="n"/>
       <c r="D12" s="7">
         <f>IF(C12="✓",$C$6,IF(C12="✗",0,""))</f>
         <v/>
@@ -767,8 +769,8 @@
     </row>
     <row r="13" ht="18" customHeight="1" s="11">
       <c r="A13" s="4" t="n"/>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="5" t="n"/>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="6" t="n"/>
       <c r="D13" s="7">
         <f>IF(C13="✓",$C$6,IF(C13="✗",0,""))</f>
         <v/>
@@ -778,8 +780,8 @@
     </row>
     <row r="14" ht="18" customHeight="1" s="11">
       <c r="A14" s="4" t="n"/>
-      <c r="B14" s="6" t="n"/>
-      <c r="C14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="6" t="n"/>
       <c r="D14" s="7">
         <f>IF(C14="✓",$C$6,IF(C14="✗",0,""))</f>
         <v/>
@@ -789,8 +791,8 @@
     </row>
     <row r="15" ht="18" customHeight="1" s="11">
       <c r="A15" s="4" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="6" t="n"/>
       <c r="D15" s="7">
         <f>IF(C15="✓",$C$6,IF(C15="✗",0,""))</f>
         <v/>
@@ -800,8 +802,8 @@
     </row>
     <row r="16" ht="18" customHeight="1" s="11">
       <c r="A16" s="4" t="n"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="5" t="n"/>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="6" t="n"/>
       <c r="D16" s="7">
         <f>IF(C16="✓",$C$6,IF(C16="✗",0,""))</f>
         <v/>
@@ -811,8 +813,8 @@
     </row>
     <row r="17" ht="18" customHeight="1" s="11">
       <c r="A17" s="4" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="5" t="n"/>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="6" t="n"/>
       <c r="D17" s="7">
         <f>IF(C17="✓",$C$6,IF(C17="✗",0,""))</f>
         <v/>
@@ -822,8 +824,8 @@
     </row>
     <row r="18" ht="18" customHeight="1" s="11">
       <c r="A18" s="4" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="5" t="n"/>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="6" t="n"/>
       <c r="D18" s="7">
         <f>IF(C18="✓",$C$6,IF(C18="✗",0,""))</f>
         <v/>
@@ -833,8 +835,8 @@
     </row>
     <row r="19" ht="18" customHeight="1" s="11">
       <c r="A19" s="4" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="5" t="n"/>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="6" t="n"/>
       <c r="D19" s="7">
         <f>IF(C19="✓",$C$6,IF(C19="✗",0,""))</f>
         <v/>
@@ -844,8 +846,8 @@
     </row>
     <row r="20" ht="18" customHeight="1" s="11">
       <c r="A20" s="4" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="5" t="n"/>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="6" t="n"/>
       <c r="D20" s="7">
         <f>IF(C20="✓",$C$6,IF(C20="✗",0,""))</f>
         <v/>
@@ -855,8 +857,8 @@
     </row>
     <row r="21" ht="18" customHeight="1" s="11">
       <c r="A21" s="4" t="n"/>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="5" t="n"/>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="6" t="n"/>
       <c r="D21" s="7">
         <f>IF(C21="✓",$C$6,IF(C21="✗",0,""))</f>
         <v/>
@@ -866,8 +868,8 @@
     </row>
     <row r="22" ht="18" customHeight="1" s="11">
       <c r="A22" s="4" t="n"/>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="5" t="n"/>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="6" t="n"/>
       <c r="D22" s="7">
         <f>IF(C22="✓",$C$6,IF(C22="✗",0,""))</f>
         <v/>
@@ -877,8 +879,8 @@
     </row>
     <row r="23" ht="18" customHeight="1" s="11">
       <c r="A23" s="4" t="n"/>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="5" t="n"/>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="6" t="n"/>
       <c r="D23" s="7">
         <f>IF(C23="✓",$C$6,IF(C23="✗",0,""))</f>
         <v/>
@@ -888,8 +890,8 @@
     </row>
     <row r="24" ht="18" customHeight="1" s="11">
       <c r="A24" s="4" t="n"/>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="5" t="n"/>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="6" t="n"/>
       <c r="D24" s="7">
         <f>IF(C24="✓",$C$6,IF(C24="✗",0,""))</f>
         <v/>
@@ -899,8 +901,8 @@
     </row>
     <row r="25" ht="18" customHeight="1" s="11">
       <c r="A25" s="4" t="n"/>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="5" t="n"/>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="6" t="n"/>
       <c r="D25" s="7">
         <f>IF(C25="✓",$C$6,IF(C25="✗",0,""))</f>
         <v/>
@@ -910,8 +912,8 @@
     </row>
     <row r="26" ht="18" customHeight="1" s="11">
       <c r="A26" s="4" t="n"/>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="5" t="n"/>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="6" t="n"/>
       <c r="D26" s="7">
         <f>IF(C26="✓",$C$6,IF(C26="✗",0,""))</f>
         <v/>
@@ -921,8 +923,8 @@
     </row>
     <row r="27" ht="18" customHeight="1" s="11">
       <c r="A27" s="4" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="5" t="n"/>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="6" t="n"/>
       <c r="D27" s="7">
         <f>IF(C27="✓",$C$6,IF(C27="✗",0,""))</f>
         <v/>

</xml_diff>